<commit_message>
fix: corrige marcas do catalogo e cadastra produtos sem marca
- Padroniza marcas no IAF (BOT/EUD/QDB/oBoticario -> canonicas)
- Corrige 18 marcas trocadas em produtos (Siage/Glam/Magnific/Pulse/Club/
  Instance/Secrets/Neo Dermo -> Eudora; 2 -> Quem Disse Berenice; OUI -> O.U.I)
- Adiciona 147 maquiagens a lista oficial iaf_make
- Cadastra 239 produtos que vinham sem marca (DESCONHECIDA) via funcao do app
- Sincroniza estoqueplanilha.xlsx e make_iaf.xlsx (fontes do rebuild) e prova
  consistencia reconstruindo o banco do zero (0 divergencias)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/estoqueplanilha.xlsx
+++ b/data/estoqueplanilha.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5236"/>
+  <dimension ref="A1:C5336"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12397,7 +12397,7 @@
       </c>
       <c r="C704" s="1" t="inlineStr">
         <is>
-          <t>OBOTICÁRIO</t>
+          <t>Quem Disse Berenice</t>
         </is>
       </c>
     </row>
@@ -78850,7 +78850,7 @@
       </c>
       <c r="C4613" s="1" t="inlineStr">
         <is>
-          <t>OBOTICÁRIO</t>
+          <t>Eudora</t>
         </is>
       </c>
     </row>
@@ -79190,7 +79190,7 @@
       </c>
       <c r="C4633" s="1" t="inlineStr">
         <is>
-          <t>OBOTICÁRIO</t>
+          <t>Eudora</t>
         </is>
       </c>
     </row>
@@ -79241,7 +79241,7 @@
       </c>
       <c r="C4636" s="1" t="inlineStr">
         <is>
-          <t>OBOTICÁRIO</t>
+          <t>Eudora</t>
         </is>
       </c>
     </row>
@@ -79428,7 +79428,7 @@
       </c>
       <c r="C4647" s="1" t="inlineStr">
         <is>
-          <t>OBOTICÁRIO</t>
+          <t>Eudora</t>
         </is>
       </c>
     </row>
@@ -79462,7 +79462,7 @@
       </c>
       <c r="C4649" s="1" t="inlineStr">
         <is>
-          <t>OBOTICÁRIO</t>
+          <t>Eudora</t>
         </is>
       </c>
     </row>
@@ -79564,7 +79564,7 @@
       </c>
       <c r="C4655" s="1" t="inlineStr">
         <is>
-          <t>OBOTICÁRIO</t>
+          <t>Eudora</t>
         </is>
       </c>
     </row>
@@ -79785,7 +79785,7 @@
       </c>
       <c r="C4668" s="1" t="inlineStr">
         <is>
-          <t>OBOTICÁRIO</t>
+          <t>Eudora</t>
         </is>
       </c>
     </row>
@@ -79887,7 +79887,7 @@
       </c>
       <c r="C4674" s="1" t="inlineStr">
         <is>
-          <t>OBOTICÁRIO</t>
+          <t>Eudora</t>
         </is>
       </c>
     </row>
@@ -79904,7 +79904,7 @@
       </c>
       <c r="C4675" s="1" t="inlineStr">
         <is>
-          <t>OBOTICÁRIO</t>
+          <t>Eudora</t>
         </is>
       </c>
     </row>
@@ -81171,7 +81171,7 @@
       <c r="B4750" s="1" t="n"/>
       <c r="C4750" s="1" t="inlineStr">
         <is>
-          <t>EUD</t>
+          <t>oBoticário</t>
         </is>
       </c>
     </row>
@@ -82663,7 +82663,7 @@
       </c>
       <c r="C4838" s="1" t="inlineStr">
         <is>
-          <t>OBOTICÁRIO</t>
+          <t>O.U.I</t>
         </is>
       </c>
     </row>
@@ -82731,7 +82731,7 @@
       </c>
       <c r="C4842" s="1" t="inlineStr">
         <is>
-          <t>OBOTICÁRIO</t>
+          <t>Quem Disse Berenice</t>
         </is>
       </c>
     </row>
@@ -85349,7 +85349,7 @@
       </c>
       <c r="C4996" s="1" t="inlineStr">
         <is>
-          <t>oBoticário</t>
+          <t>Eudora</t>
         </is>
       </c>
     </row>
@@ -85451,7 +85451,7 @@
       </c>
       <c r="C5002" s="1" t="inlineStr">
         <is>
-          <t>oBoticário</t>
+          <t>Eudora</t>
         </is>
       </c>
     </row>
@@ -85638,7 +85638,7 @@
       </c>
       <c r="C5013" s="1" t="inlineStr">
         <is>
-          <t>oBoticário</t>
+          <t>Eudora</t>
         </is>
       </c>
     </row>
@@ -85774,7 +85774,7 @@
       </c>
       <c r="C5021" s="1" t="inlineStr">
         <is>
-          <t>oBoticário</t>
+          <t>Eudora</t>
         </is>
       </c>
     </row>
@@ -85944,7 +85944,7 @@
       </c>
       <c r="C5031" s="1" t="inlineStr">
         <is>
-          <t>oBoticário</t>
+          <t>Eudora</t>
         </is>
       </c>
     </row>
@@ -86194,7 +86194,7 @@
       </c>
       <c r="B5046" t="inlineStr">
         <is>
-          <t>[EUD - VD] MÃES 2026 - COMBO INSTANCE COM ATÉ 37% DE DESCONTO</t>
+          <t>COMB INSTANCE BAUNILHA INTENSA MAES/26</t>
         </is>
       </c>
       <c r="C5046" t="inlineStr">
@@ -86216,7 +86216,7 @@
       </c>
       <c r="C5047" t="inlineStr">
         <is>
-          <t>oBoticário</t>
+          <t>Eudora</t>
         </is>
       </c>
     </row>
@@ -86432,7 +86432,7 @@
       </c>
       <c r="B5060" t="inlineStr">
         <is>
-          <t>[EUD - VD] LANÇAMENTO MÃES 2026 - COMBO BAUNILHA INTENSA COM ATÉ 21% DE DESCONTO</t>
+          <t>COMB INSTANCE BAUNILHA INTENSA MAES/26</t>
         </is>
       </c>
       <c r="C5060" t="inlineStr">
@@ -86500,7 +86500,7 @@
       </c>
       <c r="B5064" t="inlineStr">
         <is>
-          <t>COMBO MON AMIE</t>
+          <t>COMB OUI MON AMIE 037 MAES/26</t>
         </is>
       </c>
       <c r="C5064" t="inlineStr">
@@ -86828,7 +86828,7 @@
       </c>
       <c r="C5083" t="inlineStr">
         <is>
-          <t>oBoticário</t>
+          <t>Eudora</t>
         </is>
       </c>
     </row>
@@ -89430,6 +89430,1706 @@
       <c r="C5236" t="inlineStr">
         <is>
           <t>Quem Disse Berenice</t>
+        </is>
+      </c>
+    </row>
+    <row r="5237">
+      <c r="A5237" t="inlineStr">
+        <is>
+          <t>87842</t>
+        </is>
+      </c>
+      <c r="B5237" t="inlineStr">
+        <is>
+          <t>THE BLEND EDP SAFFRON 100ml</t>
+        </is>
+      </c>
+      <c r="C5237" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5238">
+      <c r="A5238" t="inlineStr">
+        <is>
+          <t>86059</t>
+        </is>
+      </c>
+      <c r="B5238" t="inlineStr">
+        <is>
+          <t>SOPHIE SPLASH CORPO E CABELO SHIMMER CHAPÉU CINTILANTE, 110ml</t>
+        </is>
+      </c>
+      <c r="C5238" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5239">
+      <c r="A5239" t="inlineStr">
+        <is>
+          <t>86058</t>
+        </is>
+      </c>
+      <c r="B5239" t="inlineStr">
+        <is>
+          <t>SOPHIE SPLASH CORPO E CABELO SHIMMER BRILHO INTERGALÁCTICO, 110ml</t>
+        </is>
+      </c>
+      <c r="C5239" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5240">
+      <c r="A5240" t="inlineStr">
+        <is>
+          <t>86061</t>
+        </is>
+      </c>
+      <c r="B5240" t="inlineStr">
+        <is>
+          <t>SOPHIE SPLASH CORPO E CABELO SHIMMER AMIZADE ILUMINADA, 110ml</t>
+        </is>
+      </c>
+      <c r="C5240" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5241">
+      <c r="A5241" t="inlineStr">
+        <is>
+          <t>90819</t>
+        </is>
+      </c>
+      <c r="B5241" t="inlineStr">
+        <is>
+          <t>SACOLA PP BOTICARIO INST/25</t>
+        </is>
+      </c>
+      <c r="C5241" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5242">
+      <c r="A5242" t="inlineStr">
+        <is>
+          <t>94969</t>
+        </is>
+      </c>
+      <c r="B5242" t="inlineStr">
+        <is>
+          <t>ROYAL LOC DES HID CPO MASC 150ml</t>
+        </is>
+      </c>
+      <c r="C5242" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5243">
+      <c r="A5243" t="inlineStr">
+        <is>
+          <t>91000</t>
+        </is>
+      </c>
+      <c r="B5243" t="inlineStr">
+        <is>
+          <t>ROYAL LOC DES HID CPO 150ml</t>
+        </is>
+      </c>
+      <c r="C5243" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5244">
+      <c r="A5244" t="inlineStr">
+        <is>
+          <t>59525</t>
+        </is>
+      </c>
+      <c r="B5244" t="inlineStr">
+        <is>
+          <t>REF NSPA LOC DES HID CPO JASM/SAMB 350ml</t>
+        </is>
+      </c>
+      <c r="C5244" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5245">
+      <c r="A5245" t="inlineStr">
+        <is>
+          <t>89203</t>
+        </is>
+      </c>
+      <c r="B5245" t="inlineStr">
+        <is>
+          <t>QUEM DISSE, BERENICE? SWEET LAB MOCHI BLUR VERMELHO GOJI BERRY, 3,5g</t>
+        </is>
+      </c>
+      <c r="C5245" t="inlineStr">
+        <is>
+          <t>Quem Disse Berenice</t>
+        </is>
+      </c>
+    </row>
+    <row r="5246">
+      <c r="A5246" t="inlineStr">
+        <is>
+          <t>89205</t>
+        </is>
+      </c>
+      <c r="B5246" t="inlineStr">
+        <is>
+          <t>QUEM DISSE, BERENICE? SWEET LAB MOCHI BLUR ROXO AMORA FUJI, 3,5g</t>
+        </is>
+      </c>
+      <c r="C5246" t="inlineStr">
+        <is>
+          <t>Quem Disse Berenice</t>
+        </is>
+      </c>
+    </row>
+    <row r="5247">
+      <c r="A5247" t="inlineStr">
+        <is>
+          <t>89206</t>
+        </is>
+      </c>
+      <c r="B5247" t="inlineStr">
+        <is>
+          <t>QUEM DISSE, BERENICE? SWEET LAB MOCHI BLUR ROSA LICHIA SAKURA, 3,5g</t>
+        </is>
+      </c>
+      <c r="C5247" t="inlineStr">
+        <is>
+          <t>Quem Disse Berenice</t>
+        </is>
+      </c>
+    </row>
+    <row r="5248">
+      <c r="A5248" t="inlineStr">
+        <is>
+          <t>89204</t>
+        </is>
+      </c>
+      <c r="B5248" t="inlineStr">
+        <is>
+          <t>QUEM DISSE, BERENICE? SWEET LAB MOCHI BLUR MARROM CACAU MATCHA, 3,5g</t>
+        </is>
+      </c>
+      <c r="C5248" t="inlineStr">
+        <is>
+          <t>Quem Disse Berenice</t>
+        </is>
+      </c>
+    </row>
+    <row r="5249">
+      <c r="A5249" t="inlineStr">
+        <is>
+          <t>90534</t>
+        </is>
+      </c>
+      <c r="B5249" t="inlineStr">
+        <is>
+          <t>QDB GLOS DOS SONHOS ROSADEX V2 4ml</t>
+        </is>
+      </c>
+      <c r="C5249" t="inlineStr">
+        <is>
+          <t>Quem Disse Berenice</t>
+        </is>
+      </c>
+    </row>
+    <row r="5250">
+      <c r="A5250" t="inlineStr">
+        <is>
+          <t>86122</t>
+        </is>
+      </c>
+      <c r="B5250" t="inlineStr">
+        <is>
+          <t>QDB BASE LIQ POP 140N 30ml</t>
+        </is>
+      </c>
+      <c r="C5250" t="inlineStr">
+        <is>
+          <t>Quem Disse Berenice</t>
+        </is>
+      </c>
+    </row>
+    <row r="5251">
+      <c r="A5251" t="inlineStr">
+        <is>
+          <t>96126</t>
+        </is>
+      </c>
+      <c r="B5251" t="inlineStr">
+        <is>
+          <t>PRESENTE NATIVA SPA QUINOA</t>
+        </is>
+      </c>
+      <c r="C5251" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5252">
+      <c r="A5252" t="inlineStr">
+        <is>
+          <t>96701</t>
+        </is>
+      </c>
+      <c r="B5252" t="inlineStr">
+        <is>
+          <t>PRESENTE CASA 214 FIGO MAGNÍFICO</t>
+        </is>
+      </c>
+      <c r="C5252" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5253">
+      <c r="A5253" t="inlineStr">
+        <is>
+          <t>94389</t>
+        </is>
+      </c>
+      <c r="B5253" t="inlineStr">
+        <is>
+          <t>PAPEL SEDA BOTI INSTIT 2025 UNIT</t>
+        </is>
+      </c>
+      <c r="C5253" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5254">
+      <c r="A5254" t="inlineStr">
+        <is>
+          <t>88623</t>
+        </is>
+      </c>
+      <c r="B5254" t="inlineStr">
+        <is>
+          <t>OUI LOC DES HID CPO LAM V2 400ml</t>
+        </is>
+      </c>
+      <c r="C5254" t="inlineStr">
+        <is>
+          <t>O.U.I</t>
+        </is>
+      </c>
+    </row>
+    <row r="5255">
+      <c r="A5255" t="inlineStr">
+        <is>
+          <t>52665</t>
+        </is>
+      </c>
+      <c r="B5255" t="inlineStr">
+        <is>
+          <t>NSPA LOC DES HID CPO F/LOT 250ml</t>
+        </is>
+      </c>
+      <c r="C5255" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5256">
+      <c r="A5256" t="inlineStr">
+        <is>
+          <t>88083</t>
+        </is>
+      </c>
+      <c r="B5256" t="inlineStr">
+        <is>
+          <t>NSPA LOC DES HID CPO AMEIX/NEG V5 200ml</t>
+        </is>
+      </c>
+      <c r="C5256" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5257">
+      <c r="A5257" t="inlineStr">
+        <is>
+          <t>88073</t>
+        </is>
+      </c>
+      <c r="B5257" t="inlineStr">
+        <is>
+          <t>NSPA CR HID MAOS AMEIXA V6 75g</t>
+        </is>
+      </c>
+      <c r="C5257" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5258">
+      <c r="A5258" t="inlineStr">
+        <is>
+          <t>90106</t>
+        </is>
+      </c>
+      <c r="B5258" t="inlineStr">
+        <is>
+          <t>NIINA SCR LAP/LAB S/PETALS C/ENCANT 0,3g</t>
+        </is>
+      </c>
+      <c r="C5258" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5259">
+      <c r="A5259" t="inlineStr">
+        <is>
+          <t>90101</t>
+        </is>
+      </c>
+      <c r="B5259" t="inlineStr">
+        <is>
+          <t>NIINA SCR BAT SFT PETALS VER/ROMAT 3,6g</t>
+        </is>
+      </c>
+      <c r="C5259" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5260">
+      <c r="A5260" t="inlineStr">
+        <is>
+          <t>90100</t>
+        </is>
+      </c>
+      <c r="B5260" t="inlineStr">
+        <is>
+          <t>NIINA SCR BAT SFT PETALS ROS SECRET 3,6g</t>
+        </is>
+      </c>
+      <c r="C5260" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5261">
+      <c r="A5261" t="inlineStr">
+        <is>
+          <t>90093</t>
+        </is>
+      </c>
+      <c r="B5261" t="inlineStr">
+        <is>
+          <t>NIINA SCR BAT SFT PETALS ROS PETALA 3,6g</t>
+        </is>
+      </c>
+      <c r="C5261" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5262">
+      <c r="A5262" t="inlineStr">
+        <is>
+          <t>90102</t>
+        </is>
+      </c>
+      <c r="B5262" t="inlineStr">
+        <is>
+          <t>NIINA SCR BAT SFT PETALS CAS/ENCANT 3,6g</t>
+        </is>
+      </c>
+      <c r="C5262" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5263">
+      <c r="A5263" t="inlineStr">
+        <is>
+          <t>59743</t>
+        </is>
+      </c>
+      <c r="B5263" t="inlineStr">
+        <is>
+          <t>NEO DERMO CR ANT FAC 30 PRO AGE V2 50g</t>
+        </is>
+      </c>
+      <c r="C5263" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5264">
+      <c r="A5264" t="inlineStr">
+        <is>
+          <t>73811</t>
+        </is>
+      </c>
+      <c r="B5264" t="inlineStr">
+        <is>
+          <t>MEN SABONETE EM BARRA, 90g C/2</t>
+        </is>
+      </c>
+      <c r="C5264" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5265">
+      <c r="A5265" t="inlineStr">
+        <is>
+          <t>90610</t>
+        </is>
+      </c>
+      <c r="B5265" t="inlineStr">
+        <is>
+          <t>MEN SAB LIQ FAC ANTIACNE 150ml</t>
+        </is>
+      </c>
+      <c r="C5265" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5266">
+      <c r="A5266" t="inlineStr">
+        <is>
+          <t>94866</t>
+        </is>
+      </c>
+      <c r="B5266" t="inlineStr">
+        <is>
+          <t>MATCH SHAMP SCIENCE RECONST V2 300ml</t>
+        </is>
+      </c>
+      <c r="C5266" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5267">
+      <c r="A5267" t="inlineStr">
+        <is>
+          <t>88895</t>
+        </is>
+      </c>
+      <c r="B5267" t="inlineStr">
+        <is>
+          <t>LIZ D'ESSENCE DESODORANTE COLÔNIA 100 ML</t>
+        </is>
+      </c>
+      <c r="C5267" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5268">
+      <c r="A5268" t="inlineStr">
+        <is>
+          <t>90298</t>
+        </is>
+      </c>
+      <c r="B5268" t="inlineStr">
+        <is>
+          <t>LIZ D'ESSENCE CREME HIDRATANTE DESODORANTE CORPORAL, 250 g</t>
+        </is>
+      </c>
+      <c r="C5268" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5269">
+      <c r="A5269" t="inlineStr">
+        <is>
+          <t>85702</t>
+        </is>
+      </c>
+      <c r="B5269" t="inlineStr">
+        <is>
+          <t>LILY EDP V3 30ml</t>
+        </is>
+      </c>
+      <c r="C5269" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5270">
+      <c r="A5270" t="inlineStr">
+        <is>
+          <t>90237</t>
+        </is>
+      </c>
+      <c r="B5270" t="inlineStr">
+        <is>
+          <t>KIT PRESENTE ZAAD PAIS 26</t>
+        </is>
+      </c>
+      <c r="C5270" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5271">
+      <c r="A5271" t="inlineStr">
+        <is>
+          <t>90242</t>
+        </is>
+      </c>
+      <c r="B5271" t="inlineStr">
+        <is>
+          <t>KIT PRESENTE UOMINI PAIS 26</t>
+        </is>
+      </c>
+      <c r="C5271" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5272">
+      <c r="A5272" t="inlineStr">
+        <is>
+          <t>89966</t>
+        </is>
+      </c>
+      <c r="B5272" t="inlineStr">
+        <is>
+          <t>Kit Presente Quasar Vision Amor 2026</t>
+        </is>
+      </c>
+      <c r="C5272" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5273">
+      <c r="A5273" t="inlineStr">
+        <is>
+          <t>90247</t>
+        </is>
+      </c>
+      <c r="B5273" t="inlineStr">
+        <is>
+          <t>KIT PRESENTE QUASAR BLUE PAIS 26</t>
+        </is>
+      </c>
+      <c r="C5273" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5274">
+      <c r="A5274" t="inlineStr">
+        <is>
+          <t>90241</t>
+        </is>
+      </c>
+      <c r="B5274" t="inlineStr">
+        <is>
+          <t>KIT PRESENTE PORTINARI PAIS 26</t>
+        </is>
+      </c>
+      <c r="C5274" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5275">
+      <c r="A5275" t="inlineStr">
+        <is>
+          <t>94440</t>
+        </is>
+      </c>
+      <c r="B5275" t="inlineStr">
+        <is>
+          <t>KIT PRESENTE OBSESSÃO POR BAUNILHA</t>
+        </is>
+      </c>
+      <c r="C5275" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5276">
+      <c r="A5276" t="inlineStr">
+        <is>
+          <t>89970</t>
+        </is>
+      </c>
+      <c r="B5276" t="inlineStr">
+        <is>
+          <t>Kit Presente Nativa Spa Orquídea Lumière Amor 2026</t>
+        </is>
+      </c>
+      <c r="C5276" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5277">
+      <c r="A5277" t="inlineStr">
+        <is>
+          <t>89958</t>
+        </is>
+      </c>
+      <c r="B5277" t="inlineStr">
+        <is>
+          <t>Kit Presente Malbec X Amor 2026</t>
+        </is>
+      </c>
+      <c r="C5277" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5278">
+      <c r="A5278" t="inlineStr">
+        <is>
+          <t>90238</t>
+        </is>
+      </c>
+      <c r="B5278" t="inlineStr">
+        <is>
+          <t>KIT PRESENTE MALBEC PAIS 26</t>
+        </is>
+      </c>
+      <c r="C5278" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5279">
+      <c r="A5279" t="inlineStr">
+        <is>
+          <t>90240</t>
+        </is>
+      </c>
+      <c r="B5279" t="inlineStr">
+        <is>
+          <t>KIT PRESENTE MALBEC ICON PAIS 26</t>
+        </is>
+      </c>
+      <c r="C5279" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5280">
+      <c r="A5280" t="inlineStr">
+        <is>
+          <t>89960</t>
+        </is>
+      </c>
+      <c r="B5280" t="inlineStr">
+        <is>
+          <t>Kit Presente L'eau de Lily Amor 2026</t>
+        </is>
+      </c>
+      <c r="C5280" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5281">
+      <c r="A5281" t="inlineStr">
+        <is>
+          <t>90253</t>
+        </is>
+      </c>
+      <c r="B5281" t="inlineStr">
+        <is>
+          <t>KIT PRESENTE KISS ME NOW</t>
+        </is>
+      </c>
+      <c r="C5281" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5282">
+      <c r="A5282" t="inlineStr">
+        <is>
+          <t>90820</t>
+        </is>
+      </c>
+      <c r="B5282" t="inlineStr">
+        <is>
+          <t>KIT PRESENTE IMENSI ALIVE</t>
+        </is>
+      </c>
+      <c r="C5282" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5283">
+      <c r="A5283" t="inlineStr">
+        <is>
+          <t>89957</t>
+        </is>
+      </c>
+      <c r="B5283" t="inlineStr">
+        <is>
+          <t>Kit Presente Her Code Climax Amor 2026</t>
+        </is>
+      </c>
+      <c r="C5283" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5284">
+      <c r="A5284" t="inlineStr">
+        <is>
+          <t>89959</t>
+        </is>
+      </c>
+      <c r="B5284" t="inlineStr">
+        <is>
+          <t>Kit Presente Floratta Red Passion Amor 2026</t>
+        </is>
+      </c>
+      <c r="C5284" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5285">
+      <c r="A5285" t="inlineStr">
+        <is>
+          <t>89963</t>
+        </is>
+      </c>
+      <c r="B5285" t="inlineStr">
+        <is>
+          <t>Kit Presente Floratta Red Amor 2026</t>
+        </is>
+      </c>
+      <c r="C5285" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5286">
+      <c r="A5286" t="inlineStr">
+        <is>
+          <t>90250</t>
+        </is>
+      </c>
+      <c r="B5286" t="inlineStr">
+        <is>
+          <t>KIT PRESENTE EGEO ORIGINAL PAIS 26</t>
+        </is>
+      </c>
+      <c r="C5286" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5287">
+      <c r="A5287" t="inlineStr">
+        <is>
+          <t>89964</t>
+        </is>
+      </c>
+      <c r="B5287" t="inlineStr">
+        <is>
+          <t>Kit Presente Egeo Dolce Amor 2026</t>
+        </is>
+      </c>
+      <c r="C5287" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5288">
+      <c r="A5288" t="inlineStr">
+        <is>
+          <t>89965</t>
+        </is>
+      </c>
+      <c r="B5288" t="inlineStr">
+        <is>
+          <t>Kit Presente Egeo Bomb Black Amor 2026</t>
+        </is>
+      </c>
+      <c r="C5288" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5289">
+      <c r="A5289" t="inlineStr">
+        <is>
+          <t>89969</t>
+        </is>
+      </c>
+      <c r="B5289" t="inlineStr">
+        <is>
+          <t>Kit Presente Cuide-se Bem Amoruda Amor 2026</t>
+        </is>
+      </c>
+      <c r="C5289" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5290">
+      <c r="A5290" t="inlineStr">
+        <is>
+          <t>94630</t>
+        </is>
+      </c>
+      <c r="B5290" t="inlineStr">
+        <is>
+          <t>KIT PRESENTE CONNEXION PAIS 26</t>
+        </is>
+      </c>
+      <c r="C5290" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5291">
+      <c r="A5291" t="inlineStr">
+        <is>
+          <t>89962</t>
+        </is>
+      </c>
+      <c r="B5291" t="inlineStr">
+        <is>
+          <t>Kit Presente Coffee Woman Sedution Amor 2026</t>
+        </is>
+      </c>
+      <c r="C5291" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5292">
+      <c r="A5292" t="inlineStr">
+        <is>
+          <t>94441</t>
+        </is>
+      </c>
+      <c r="B5292" t="inlineStr">
+        <is>
+          <t>KIT PRESENTE CLUB 6</t>
+        </is>
+      </c>
+      <c r="C5292" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5293">
+      <c r="A5293" t="inlineStr">
+        <is>
+          <t>90243</t>
+        </is>
+      </c>
+      <c r="B5293" t="inlineStr">
+        <is>
+          <t>KIT PRESENTE CLASH PAIS 26</t>
+        </is>
+      </c>
+      <c r="C5293" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5294">
+      <c r="A5294" t="inlineStr">
+        <is>
+          <t>90852</t>
+        </is>
+      </c>
+      <c r="B5294" t="inlineStr">
+        <is>
+          <t>KIT PRESENTE CELEBRE SUA FORÇA PAIS 26</t>
+        </is>
+      </c>
+      <c r="C5294" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5295">
+      <c r="A5295" t="inlineStr">
+        <is>
+          <t>89967</t>
+        </is>
+      </c>
+      <c r="B5295" t="inlineStr">
+        <is>
+          <t>Kit Presente Celebre Agora MAsculino Amor 2026</t>
+        </is>
+      </c>
+      <c r="C5295" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5296">
+      <c r="A5296" t="inlineStr">
+        <is>
+          <t>89968</t>
+        </is>
+      </c>
+      <c r="B5296" t="inlineStr">
+        <is>
+          <t>Kit Presente Celebre Agora Feminino Amor 2026</t>
+        </is>
+      </c>
+      <c r="C5296" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5297">
+      <c r="A5297" t="inlineStr">
+        <is>
+          <t>89961</t>
+        </is>
+      </c>
+      <c r="B5297" t="inlineStr">
+        <is>
+          <t>Kit Presente Botica 214 Dark Mint Amor 2026</t>
+        </is>
+      </c>
+      <c r="C5297" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5298">
+      <c r="A5298" t="inlineStr">
+        <is>
+          <t>90255</t>
+        </is>
+      </c>
+      <c r="B5298" t="inlineStr">
+        <is>
+          <t>KIT PRESENTE BODY SPRAY IMPRESSION E INTENTION</t>
+        </is>
+      </c>
+      <c r="C5298" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5299">
+      <c r="A5299" t="inlineStr">
+        <is>
+          <t>90239</t>
+        </is>
+      </c>
+      <c r="B5299" t="inlineStr">
+        <is>
+          <t>KIT PRESENTE ARBO PAIS 26</t>
+        </is>
+      </c>
+      <c r="C5299" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5300">
+      <c r="A5300" t="inlineStr">
+        <is>
+          <t>90902</t>
+        </is>
+      </c>
+      <c r="B5300" t="inlineStr">
+        <is>
+          <t>KIT DR BOTICA MAGICO TEATRO BONECOS V2</t>
+        </is>
+      </c>
+      <c r="C5300" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5301">
+      <c r="A5301" t="inlineStr">
+        <is>
+          <t>91302</t>
+        </is>
+      </c>
+      <c r="B5301" t="inlineStr">
+        <is>
+          <t>INSTANCE DES COL FR/VERM 200ml</t>
+        </is>
+      </c>
+      <c r="C5301" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5302">
+      <c r="A5302" t="inlineStr">
+        <is>
+          <t>95619</t>
+        </is>
+      </c>
+      <c r="B5302" t="inlineStr">
+        <is>
+          <t>INSTANCE D/COL BDY/SPL MOR/IRR V2 200ml</t>
+        </is>
+      </c>
+      <c r="C5302" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5303">
+      <c r="A5303" t="inlineStr">
+        <is>
+          <t>95353</t>
+        </is>
+      </c>
+      <c r="B5303" t="inlineStr">
+        <is>
+          <t>INSTANCE CR DES H CP AMEIX/PR 180ml RPCK</t>
+        </is>
+      </c>
+      <c r="C5303" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5304">
+      <c r="A5304" t="inlineStr">
+        <is>
+          <t>85955</t>
+        </is>
+      </c>
+      <c r="B5304" t="inlineStr">
+        <is>
+          <t>INSTANCE CALDA BNH AMEIX/PRAL RPKC 180ml</t>
+        </is>
+      </c>
+      <c r="C5304" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5305">
+      <c r="A5305" t="inlineStr">
+        <is>
+          <t>84874</t>
+        </is>
+      </c>
+      <c r="B5305" t="inlineStr">
+        <is>
+          <t>EUD MAKE BAT MATE K/M ROS/UNICO V4 3,7g</t>
+        </is>
+      </c>
+      <c r="C5305" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5306">
+      <c r="A5306" t="inlineStr">
+        <is>
+          <t>89767</t>
+        </is>
+      </c>
+      <c r="B5306" t="inlineStr">
+        <is>
+          <t>EUD DES COL VELVET SOUL 100ml</t>
+        </is>
+      </c>
+      <c r="C5306" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5307">
+      <c r="A5307" t="inlineStr">
+        <is>
+          <t>90141</t>
+        </is>
+      </c>
+      <c r="B5307" t="inlineStr">
+        <is>
+          <t>EUD DES BDY SPR VELVET SOUL 100ml</t>
+        </is>
+      </c>
+      <c r="C5307" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5308">
+      <c r="A5308" t="inlineStr">
+        <is>
+          <t>52654</t>
+        </is>
+      </c>
+      <c r="B5308" t="inlineStr">
+        <is>
+          <t>ESTJ NSPA QUINOA REG/21 V2</t>
+        </is>
+      </c>
+      <c r="C5308" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5309">
+      <c r="A5309" t="inlineStr">
+        <is>
+          <t>94400</t>
+        </is>
+      </c>
+      <c r="B5309" t="inlineStr">
+        <is>
+          <t>ESTJ CASA 214 FIGO MAGNIFICO</t>
+        </is>
+      </c>
+      <c r="C5309" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5310">
+      <c r="A5310" t="inlineStr">
+        <is>
+          <t>81264</t>
+        </is>
+      </c>
+      <c r="B5310" t="inlineStr">
+        <is>
+          <t>DEM CBEM DES COL BDY SPLSH BEND/CACT 4ml</t>
+        </is>
+      </c>
+      <c r="C5310" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5311">
+      <c r="A5311" t="inlineStr">
+        <is>
+          <t>85654</t>
+        </is>
+      </c>
+      <c r="B5311" t="inlineStr">
+        <is>
+          <t>DEM BOTICA 214 EDP ARAB/OAS FL/FRUT 4ml</t>
+        </is>
+      </c>
+      <c r="C5311" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5312">
+      <c r="A5312" t="inlineStr">
+        <is>
+          <t>89397</t>
+        </is>
+      </c>
+      <c r="B5312" t="inlineStr">
+        <is>
+          <t>CX PRESENTE G BOT INST/25 VDA</t>
+        </is>
+      </c>
+      <c r="C5312" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5313">
+      <c r="A5313" t="inlineStr">
+        <is>
+          <t>98403</t>
+        </is>
+      </c>
+      <c r="B5313" t="inlineStr">
+        <is>
+          <t>COMBO SIAGE NUTRI DIAMOND (5 itens)</t>
+        </is>
+      </c>
+      <c r="C5313" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5314">
+      <c r="A5314" t="inlineStr">
+        <is>
+          <t>96462</t>
+        </is>
+      </c>
+      <c r="B5314" t="inlineStr">
+        <is>
+          <t>COMBO SIAGE NUTRI DIAMOND (3 itens)</t>
+        </is>
+      </c>
+      <c r="C5314" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5315">
+      <c r="A5315" t="inlineStr">
+        <is>
+          <t>97991</t>
+        </is>
+      </c>
+      <c r="B5315" t="inlineStr">
+        <is>
+          <t>COMBO SIAGE NUTRI DIAMOND (2 itens)</t>
+        </is>
+      </c>
+      <c r="C5315" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5316">
+      <c r="A5316" t="inlineStr">
+        <is>
+          <t>97852</t>
+        </is>
+      </c>
+      <c r="B5316" t="inlineStr">
+        <is>
+          <t>Combo Siage Acelera o Crescimento (4 Itens)</t>
+        </is>
+      </c>
+      <c r="C5316" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5317">
+      <c r="A5317" t="inlineStr">
+        <is>
+          <t>98399</t>
+        </is>
+      </c>
+      <c r="B5317" t="inlineStr">
+        <is>
+          <t>COMBO MATCH</t>
+        </is>
+      </c>
+      <c r="C5317" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5318">
+      <c r="A5318" t="inlineStr">
+        <is>
+          <t>98196</t>
+        </is>
+      </c>
+      <c r="B5318" t="inlineStr">
+        <is>
+          <t>COMBO LILY ( 2 ITENS)</t>
+        </is>
+      </c>
+      <c r="C5318" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5319">
+      <c r="A5319" t="inlineStr">
+        <is>
+          <t>98400</t>
+        </is>
+      </c>
+      <c r="B5319" t="inlineStr">
+        <is>
+          <t>COMB SOPHIE SHIMMER</t>
+        </is>
+      </c>
+      <c r="C5319" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5320">
+      <c r="A5320" t="inlineStr">
+        <is>
+          <t>96468</t>
+        </is>
+      </c>
+      <c r="B5320" t="inlineStr">
+        <is>
+          <t>COMB SIAGE VOLUME IMEDIATO 02</t>
+        </is>
+      </c>
+      <c r="C5320" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5321">
+      <c r="A5321" t="inlineStr">
+        <is>
+          <t>96461</t>
+        </is>
+      </c>
+      <c r="B5321" t="inlineStr">
+        <is>
+          <t>COMB SIAGE PRO CRONOLOGY CURVAS 03</t>
+        </is>
+      </c>
+      <c r="C5321" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5322">
+      <c r="A5322" t="inlineStr">
+        <is>
+          <t>96078</t>
+        </is>
+      </c>
+      <c r="B5322" t="inlineStr">
+        <is>
+          <t>COMB QDB 03 MAES/26</t>
+        </is>
+      </c>
+      <c r="C5322" t="inlineStr">
+        <is>
+          <t>Quem Disse Berenice</t>
+        </is>
+      </c>
+    </row>
+    <row r="5323">
+      <c r="A5323" t="inlineStr">
+        <is>
+          <t>96374</t>
+        </is>
+      </c>
+      <c r="B5323" t="inlineStr">
+        <is>
+          <t>COMB OUI SCAPIN 245 02 MAES/26</t>
+        </is>
+      </c>
+      <c r="C5323" t="inlineStr">
+        <is>
+          <t>O.U.I</t>
+        </is>
+      </c>
+    </row>
+    <row r="5324">
+      <c r="A5324" t="inlineStr">
+        <is>
+          <t>95916</t>
+        </is>
+      </c>
+      <c r="B5324" t="inlineStr">
+        <is>
+          <t>COMB LA VICTORIE AMOR/26</t>
+        </is>
+      </c>
+      <c r="C5324" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5325">
+      <c r="A5325" t="inlineStr">
+        <is>
+          <t>95696</t>
+        </is>
+      </c>
+      <c r="B5325" t="inlineStr">
+        <is>
+          <t>COMB EUDORA H MARINE NAM/26</t>
+        </is>
+      </c>
+      <c r="C5325" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5326">
+      <c r="A5326" t="inlineStr">
+        <is>
+          <t>96819</t>
+        </is>
+      </c>
+      <c r="B5326" t="inlineStr">
+        <is>
+          <t>COMB EUD VELVET SOUL 02</t>
+        </is>
+      </c>
+      <c r="C5326" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5327">
+      <c r="A5327" t="inlineStr">
+        <is>
+          <t>96818</t>
+        </is>
+      </c>
+      <c r="B5327" t="inlineStr">
+        <is>
+          <t>COMB EUD VELVET SOUL</t>
+        </is>
+      </c>
+      <c r="C5327" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5328">
+      <c r="A5328" t="inlineStr">
+        <is>
+          <t>95695</t>
+        </is>
+      </c>
+      <c r="B5328" t="inlineStr">
+        <is>
+          <t>COMB EUD ROUGE NAM/26</t>
+        </is>
+      </c>
+      <c r="C5328" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5329">
+      <c r="A5329" t="inlineStr">
+        <is>
+          <t>97594</t>
+        </is>
+      </c>
+      <c r="B5329" t="inlineStr">
+        <is>
+          <t>COMB DIVA SUPREMA AMOR/26</t>
+        </is>
+      </c>
+      <c r="C5329" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5330">
+      <c r="A5330" t="inlineStr">
+        <is>
+          <t>95913</t>
+        </is>
+      </c>
+      <c r="B5330" t="inlineStr">
+        <is>
+          <t>COMB CLUB 6 CASSINO AMOR/26</t>
+        </is>
+      </c>
+      <c r="C5330" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5331">
+      <c r="A5331" t="inlineStr">
+        <is>
+          <t>98401</t>
+        </is>
+      </c>
+      <c r="B5331" t="inlineStr">
+        <is>
+          <t>COMB CBEM DES COL BODY SPLASH 1</t>
+        </is>
+      </c>
+      <c r="C5331" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5332">
+      <c r="A5332" t="inlineStr">
+        <is>
+          <t>98402</t>
+        </is>
+      </c>
+      <c r="B5332" t="inlineStr">
+        <is>
+          <t>COMB CBEM BODY SPLASH 2</t>
+        </is>
+      </c>
+      <c r="C5332" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5333">
+      <c r="A5333" t="inlineStr">
+        <is>
+          <t>98191</t>
+        </is>
+      </c>
+      <c r="B5333" t="inlineStr">
+        <is>
+          <t>COMB BOTICA 214 ARABIAN OASIS (4 itens)</t>
+        </is>
+      </c>
+      <c r="C5333" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5334">
+      <c r="A5334" t="inlineStr">
+        <is>
+          <t>94676</t>
+        </is>
+      </c>
+      <c r="B5334" t="inlineStr">
+        <is>
+          <t>CBEM ESF FAC FEIRA MORANGO V2 100g</t>
+        </is>
+      </c>
+      <c r="C5334" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5335">
+      <c r="A5335" t="inlineStr">
+        <is>
+          <t>85645</t>
+        </is>
+      </c>
+      <c r="B5335" t="inlineStr">
+        <is>
+          <t>BOTICA 214 ARABIAN OASIS FOUGÈRE AMBARADO EAU DE PARFUM, 90ml</t>
+        </is>
+      </c>
+      <c r="C5335" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5336">
+      <c r="A5336" t="inlineStr">
+        <is>
+          <t>85644</t>
+        </is>
+      </c>
+      <c r="B5336" t="inlineStr">
+        <is>
+          <t>BOTICA 214 ARABIAN OASIS FLORAL FRUTAL EAU DE PARFUM, 75ml</t>
+        </is>
+      </c>
+      <c r="C5336" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(catalogo): cadastra 22 produtos do grupo que caiam sem marca
Produtos vendidos (base Platina/Penedo) que nao existiam no catalogo e
viravam DESCONHECIDA: Club 6, Impression, Niina, Eud Make (Eudora);
Cuide-se Bem, Malbec, Coffee, Liz, Nspa, Her Code (oBoticario); Desir
(O.U.I). Marcas confirmadas por evidencia do proprio catalogo + usuario.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/estoqueplanilha.xlsx
+++ b/data/estoqueplanilha.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5336"/>
+  <dimension ref="A1:C5358"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -91130,6 +91130,380 @@
       <c r="C5336" t="inlineStr">
         <is>
           <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5337">
+      <c r="A5337" t="inlineStr">
+        <is>
+          <t>97395</t>
+        </is>
+      </c>
+      <c r="B5337" t="inlineStr">
+        <is>
+          <t>COMB CLUB 6 PRESTIGE PAIS/26</t>
+        </is>
+      </c>
+      <c r="C5337" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5338">
+      <c r="A5338" t="inlineStr">
+        <is>
+          <t>87938</t>
+        </is>
+      </c>
+      <c r="B5338" t="inlineStr">
+        <is>
+          <t>CLUB 6 EAU DE PARFUM, 95 ml</t>
+        </is>
+      </c>
+      <c r="C5338" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5339">
+      <c r="A5339" t="inlineStr">
+        <is>
+          <t>96809</t>
+        </is>
+      </c>
+      <c r="B5339" t="inlineStr">
+        <is>
+          <t>COMB IMPRESSION PAIS/26</t>
+        </is>
+      </c>
+      <c r="C5339" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5340">
+      <c r="A5340" t="inlineStr">
+        <is>
+          <t>94163</t>
+        </is>
+      </c>
+      <c r="B5340" t="inlineStr">
+        <is>
+          <t>NIINA SCRT PLT SOMBRAS SOFT PETALS 10g</t>
+        </is>
+      </c>
+      <c r="C5340" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5341">
+      <c r="A5341" t="inlineStr">
+        <is>
+          <t>96805</t>
+        </is>
+      </c>
+      <c r="B5341" t="inlineStr">
+        <is>
+          <t>COMB EUDORA H ACQUA PAIS/26</t>
+        </is>
+      </c>
+      <c r="C5341" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5342">
+      <c r="A5342" t="inlineStr">
+        <is>
+          <t>98542</t>
+        </is>
+      </c>
+      <c r="B5342" t="inlineStr">
+        <is>
+          <t>COMB NIINA SECRETS SOFT PETALS 03</t>
+        </is>
+      </c>
+      <c r="C5342" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5343">
+      <c r="A5343" t="inlineStr">
+        <is>
+          <t>96804</t>
+        </is>
+      </c>
+      <c r="B5343" t="inlineStr">
+        <is>
+          <t>COMB EUD SENSUAL VELVET PAIS/26</t>
+        </is>
+      </c>
+      <c r="C5343" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5344">
+      <c r="A5344" t="inlineStr">
+        <is>
+          <t>95312</t>
+        </is>
+      </c>
+      <c r="B5344" t="inlineStr">
+        <is>
+          <t>NIINA SCR BAT SFT PETALS MAR/AVELUD 3,6g</t>
+        </is>
+      </c>
+      <c r="C5344" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5345">
+      <c r="A5345" t="inlineStr">
+        <is>
+          <t>84872</t>
+        </is>
+      </c>
+      <c r="B5345" t="inlineStr">
+        <is>
+          <t>EUD MAKE BATOM MATTE KISS ME NUDE REALCE</t>
+        </is>
+      </c>
+      <c r="C5345" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5346">
+      <c r="A5346" t="inlineStr">
+        <is>
+          <t>90103</t>
+        </is>
+      </c>
+      <c r="B5346" t="inlineStr">
+        <is>
+          <t>NIINA SCR LAP/LAB S/PETALS R/PETALA 0,3g</t>
+        </is>
+      </c>
+      <c r="C5346" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5347">
+      <c r="A5347" t="inlineStr">
+        <is>
+          <t>90105</t>
+        </is>
+      </c>
+      <c r="B5347" t="inlineStr">
+        <is>
+          <t>NIINA SCR LAP/LAB S/PETALS VER/ROM 0,3g</t>
+        </is>
+      </c>
+      <c r="C5347" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5348">
+      <c r="A5348" t="inlineStr">
+        <is>
+          <t>95313</t>
+        </is>
+      </c>
+      <c r="B5348" t="inlineStr">
+        <is>
+          <t>NIINA SCR LAP/LAB S/PETALS MAR/AVEL 0,3g</t>
+        </is>
+      </c>
+      <c r="C5348" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+    </row>
+    <row r="5349">
+      <c r="A5349" t="inlineStr">
+        <is>
+          <t>88688</t>
+        </is>
+      </c>
+      <c r="B5349" t="inlineStr">
+        <is>
+          <t>CBEM LOC DES HID CPO NUVEM N/FORM 400ml</t>
+        </is>
+      </c>
+      <c r="C5349" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5350">
+      <c r="A5350" t="inlineStr">
+        <is>
+          <t>86798</t>
+        </is>
+      </c>
+      <c r="B5350" t="inlineStr">
+        <is>
+          <t>NSPA CR PARFUMEE CPO AMEIXA 200g</t>
+        </is>
+      </c>
+      <c r="C5350" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5351">
+      <c r="A5351" t="inlineStr">
+        <is>
+          <t>95648</t>
+        </is>
+      </c>
+      <c r="B5351" t="inlineStr">
+        <is>
+          <t>KIT PRESENTE COFFEE MAN ADDICTIVE PAIS 26</t>
+        </is>
+      </c>
+      <c r="C5351" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5352">
+      <c r="A5352" t="inlineStr">
+        <is>
+          <t>90249</t>
+        </is>
+      </c>
+      <c r="B5352" t="inlineStr">
+        <is>
+          <t>KIT PRESENTE MALBEC B/SPRAY PAIS 26</t>
+        </is>
+      </c>
+      <c r="C5352" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5353">
+      <c r="A5353" t="inlineStr">
+        <is>
+          <t>94499</t>
+        </is>
+      </c>
+      <c r="B5353" t="inlineStr">
+        <is>
+          <t>CBEM SAB BARRA PESSEGURA V3 4x80g</t>
+        </is>
+      </c>
+      <c r="C5353" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5354">
+      <c r="A5354" t="inlineStr">
+        <is>
+          <t>88130</t>
+        </is>
+      </c>
+      <c r="B5354" t="inlineStr">
+        <is>
+          <t>HER CODE BODY SPLASH DESODORANTE COLONIA, 200ml</t>
+        </is>
+      </c>
+      <c r="C5354" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5355">
+      <c r="A5355" t="inlineStr">
+        <is>
+          <t>88971</t>
+        </is>
+      </c>
+      <c r="B5355" t="inlineStr">
+        <is>
+          <t>LIZ DES COL D ESSENCE PRM 10ml</t>
+        </is>
+      </c>
+      <c r="C5355" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5356">
+      <c r="A5356" t="inlineStr">
+        <is>
+          <t>85653</t>
+        </is>
+      </c>
+      <c r="B5356" t="inlineStr">
+        <is>
+          <t>DEM BOTICA 214 EDP ARAB/OAS FOUG/AMB 4ml</t>
+        </is>
+      </c>
+      <c r="C5356" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5357">
+      <c r="A5357" t="inlineStr">
+        <is>
+          <t>88897</t>
+        </is>
+      </c>
+      <c r="B5357" t="inlineStr">
+        <is>
+          <t>CJ FLAC LIZ DES COL D ESSENCE 5x1ml</t>
+        </is>
+      </c>
+      <c r="C5357" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+    </row>
+    <row r="5358">
+      <c r="A5358" t="inlineStr">
+        <is>
+          <t>86396</t>
+        </is>
+      </c>
+      <c r="B5358" t="inlineStr">
+        <is>
+          <t>O.U.i Desir Parisien 750 Eau de Parfum Pour Femme 75ml</t>
+        </is>
+      </c>
+      <c r="C5358" t="inlineStr">
+        <is>
+          <t>O.U.I</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(catalogo): corrige marca Instance/Niina (Eudora cadastrada como oBoticario)
7 SKUs da linha Eudora estavam cadastrados como oBoticario, colapsando duas
marcas numa so e SUBcontando multimarca:
- Instance (6 SKUs: cremes de maos / locoes corporais)
- Niina Secrets Hair Clip (1 SKU)

Efeito (so positivo, nenhum multimarca falso removido): +8 clientes multimarca
no arquivo de Platina (Platina/Penedo 47->48, alem de Ouro, Prata 3 e FVC).
Chega em producao no proximo deploy via UPSERT do import_produtos.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/estoqueplanilha.xlsx
+++ b/data/estoqueplanilha.xlsx
@@ -78748,7 +78748,7 @@
       </c>
       <c r="C4607" s="1" t="inlineStr">
         <is>
-          <t>OBOTICÁRIO</t>
+          <t>Eudora</t>
         </is>
       </c>
     </row>
@@ -78935,7 +78935,7 @@
       </c>
       <c r="C4618" s="1" t="inlineStr">
         <is>
-          <t>OBOTICÁRIO</t>
+          <t>Eudora</t>
         </is>
       </c>
     </row>
@@ -79921,7 +79921,7 @@
       </c>
       <c r="C4676" s="1" t="inlineStr">
         <is>
-          <t>OBOTICÁRIO</t>
+          <t>Eudora</t>
         </is>
       </c>
     </row>
@@ -79955,7 +79955,7 @@
       </c>
       <c r="C4678" s="1" t="inlineStr">
         <is>
-          <t>OBOTICÁRIO</t>
+          <t>Eudora</t>
         </is>
       </c>
     </row>
@@ -82935,7 +82935,7 @@
       </c>
       <c r="C4854" s="1" t="inlineStr">
         <is>
-          <t>OBOTICÁRIO</t>
+          <t>Eudora</t>
         </is>
       </c>
     </row>
@@ -83003,7 +83003,7 @@
       </c>
       <c r="C4858" s="1" t="inlineStr">
         <is>
-          <t>OBOTICÁRIO</t>
+          <t>Eudora</t>
         </is>
       </c>
     </row>
@@ -83190,7 +83190,7 @@
       </c>
       <c r="C4869" s="1" t="inlineStr">
         <is>
-          <t>OBOTICÁRIO</t>
+          <t>Eudora</t>
         </is>
       </c>
     </row>

</xml_diff>